<commit_message>
fix(onboarding): PUNTO 3 · bloque contratos (#1413)
Ida y vuelta del flujo (?from=empezar) + cierre del bucle + off-by-one de fechas + plantilla ATLAS espejo del wizard (columnas opcionales retrocompatibles) + importador en 3 pasos con autodetección por cabecera. Atendidos los 3 comentarios de Copilot.
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-contratos-atlas.xlsx
+++ b/public/templates/plantilla-contratos-atlas.xlsx
@@ -32,8 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+    <numFmt numFmtId="60" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -64,8 +65,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,20 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="17.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:O4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -446,6 +435,18 @@
       <c r="K1" t="str">
         <v>Fianza €</v>
       </c>
+      <c r="L1" t="str">
+        <v>Día de pago</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Indexación</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Reducción IRPF %</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Cotitulares (NIFs)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -457,11 +458,11 @@
       <c r="C2" t="str">
         <v>Vivienda LAU</v>
       </c>
-      <c r="D2" t="str">
-        <v>01/01/2024</v>
-      </c>
-      <c r="E2" t="str">
-        <v>31/12/2028</v>
+      <c r="D2" s="1">
+        <v>45292</v>
+      </c>
+      <c r="E2" s="1">
+        <v>47118</v>
       </c>
       <c r="F2" t="str">
         <v>CONCEPCION RAMIREZ GUERERO</v>
@@ -480,6 +481,18 @@
       </c>
       <c r="K2">
         <v>330</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2" t="str">
+        <v>IPC anual</v>
+      </c>
+      <c r="N2">
+        <v>60</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -492,8 +505,8 @@
       <c r="C3" t="str">
         <v>Vivienda LAU</v>
       </c>
-      <c r="D3" t="str">
-        <v>01/02/2024</v>
+      <c r="D3" s="1">
+        <v>45323</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -515,6 +528,18 @@
       </c>
       <c r="K3">
         <v>600</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Sin indexación</v>
+      </c>
+      <c r="N3">
+        <v>50</v>
+      </c>
+      <c r="O3" t="str">
+        <v>12345678Z</v>
       </c>
     </row>
     <row r="4">
@@ -527,11 +552,11 @@
       <c r="C4" t="str">
         <v>Vacacional</v>
       </c>
-      <c r="D4" t="str">
-        <v>01/07/2024</v>
-      </c>
-      <c r="E4" t="str">
-        <v>31/08/2024</v>
+      <c r="D4" s="1">
+        <v>45474</v>
+      </c>
+      <c r="E4" s="1">
+        <v>45535</v>
       </c>
       <c r="F4" t="str">
         <v>FAMILIA MARTINEZ</v>
@@ -550,11 +575,23 @@
       </c>
       <c r="K4">
         <v>0</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>